<commit_message>
Add GST and attachment findings to the September card checks
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RHXHFGjwTVGyoJeP29asg9
</commit_message>
<xml_diff>
--- a/cards/09. DL CTS EXP SEPT 26.xlsx
+++ b/cards/09. DL CTS EXP SEPT 26.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="43">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -52,6 +52,9 @@
     <t xml:space="preserve">CTS 20th Anniversary team lunch</t>
   </si>
   <si>
+    <t xml:space="preserve">In Xero. Bill name says paid via PL CC but it was paid from the DL card. Label only.</t>
+  </si>
+  <si>
     <t xml:space="preserve">BARISTA VS CHEF          Sydney      NSW</t>
   </si>
   <si>
@@ -82,6 +85,9 @@
     <t xml:space="preserve">BL Apple iCLoud Storage (Duncan's daughter's)</t>
   </si>
   <si>
+    <t xml:space="preserve">In Xero but no invoice attached.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Spacera Sales Lunch Meeting</t>
   </si>
   <si>
@@ -122,6 +128,9 @@
   </si>
   <si>
     <t xml:space="preserve">DEWR Lunch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In Xero. The CTS half of the lunch (32.00) has no GST on it but the DEWR half does. Minor, 2.91.</t>
   </si>
   <si>
     <t xml:space="preserve">CAFE RISTRETTO           CANBERRA    ACT</t>
@@ -146,11 +155,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* \-??_);_(@_)"/>
-    <numFmt numFmtId="166" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* \-??_-;_-@_-"/>
-    <numFmt numFmtId="167" formatCode="m/d/yyyy"/>
+    <numFmt numFmtId="165" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* \-??_-;_-@_-"/>
+    <numFmt numFmtId="166" formatCode="m/d/yyyy"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -251,25 +259,26 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="15" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -277,31 +286,27 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="15" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="2" borderId="0" xfId="15" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -309,11 +314,15 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -570,350 +579,365 @@
   <sheetFormatPr defaultColWidth="8.53125" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="48.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="12.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="76.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="10.4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="48.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="3" width="12.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="76.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="10.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="70"/>
   </cols>
   <sheetData>
-    <row r="1" s="4" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="3" t="s">
+    <row r="1" s="5" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="7" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="7" t="n">
+    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="8" t="n">
         <v>46269</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="9" t="n">
+      <c r="C2" s="10" t="n">
         <v>-46.6</v>
       </c>
-      <c r="D2" s="10" t="s">
+      <c r="D2" s="2" t="s">
         <v>6</v>
       </c>
       <c r="E2" s="11" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="7" t="n">
+    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="8" t="n">
         <v>46271</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="9" t="n">
+      <c r="C3" s="10" t="n">
         <v>-1099</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="D3" s="2" t="s">
         <v>9</v>
       </c>
       <c r="E3" s="11" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="12" t="n">
+      <c r="F3" s="12" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="13" t="n">
         <v>46273</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>-30.96</v>
+      </c>
+      <c r="F4" s="14" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="13" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>-25.65</v>
+      </c>
+      <c r="F5" s="14" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="8" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="10" t="n">
+        <v>-54.57</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="13" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>-15.16</v>
+      </c>
+      <c r="F7" s="14" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="8" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" s="10" t="n">
+        <v>-41.82</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E8" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="F8" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="2" t="n">
-        <v>-30.96</v>
-      </c>
-      <c r="F4" s="13" t="s">
+    </row>
+    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="8" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" s="10" t="n">
+        <v>-14.99</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E9" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="F9" s="12" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="8" t="n">
+        <v>46289</v>
+      </c>
+      <c r="B10" s="9" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="12" t="n">
-        <v>46276</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" s="2" t="n">
-        <v>-25.65</v>
-      </c>
-      <c r="F5" s="13" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="n">
-        <v>46281</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" s="9" t="n">
-        <v>-54.57</v>
-      </c>
-      <c r="D6" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="E6" s="11" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="12" t="n">
-        <v>46281</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="C7" s="2" t="n">
-        <v>-15.16</v>
-      </c>
-      <c r="F7" s="13" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="n">
+      <c r="C10" s="10" t="n">
+        <v>-56.84</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E10" s="11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="8" t="n">
         <v>46289</v>
       </c>
-      <c r="B8" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" s="9" t="n">
-        <v>-41.82</v>
-      </c>
-      <c r="D8" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="E8" s="11" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="n">
-        <v>46289</v>
-      </c>
-      <c r="B9" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="C9" s="9" t="n">
-        <v>-14.99</v>
-      </c>
-      <c r="D9" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="E9" s="11" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="n">
-        <v>46289</v>
-      </c>
-      <c r="B10" s="8" t="s">
+      <c r="B11" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="C11" s="10" t="n">
+        <v>-15.86</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E11" s="11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="8" t="n">
+        <v>46290</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" s="10" t="n">
+        <v>-171.94</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E12" s="11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="8" t="n">
+        <v>46292</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C13" s="10" t="n">
+        <v>-257.81</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E13" s="11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="8" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="C14" s="10" t="n">
+        <v>-49.61</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E14" s="11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="8" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="C15" s="10" t="n">
+        <v>-20</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="E15" s="11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="8" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C16" s="10" t="n">
+        <v>-16.99</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E16" s="11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="8" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="C17" s="10" t="n">
+        <v>-65.02</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E17" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="F17" s="12" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="8" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B18" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="C18" s="10" t="n">
+        <v>-12.8</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E18" s="11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="8" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="C19" s="10" t="n">
+        <v>-43.74</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="E19" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="F19" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="9" t="n">
-        <v>-56.84</v>
-      </c>
-      <c r="D10" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="E10" s="11" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="7" t="n">
-        <v>46289</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="C11" s="9" t="n">
-        <v>-15.86</v>
-      </c>
-      <c r="D11" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="E11" s="11" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="7" t="n">
-        <v>46290</v>
-      </c>
-      <c r="B12" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="C12" s="9" t="n">
-        <v>-171.94</v>
-      </c>
-      <c r="D12" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="E12" s="11" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="7" t="n">
-        <v>46292</v>
-      </c>
-      <c r="B13" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="C13" s="9" t="n">
-        <v>-257.81</v>
-      </c>
-      <c r="D13" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="E13" s="11" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="7" t="n">
-        <v>46293</v>
-      </c>
-      <c r="B14" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="C14" s="9" t="n">
-        <v>-49.61</v>
-      </c>
-      <c r="D14" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="E14" s="11" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="7" t="n">
-        <v>46293</v>
-      </c>
-      <c r="B15" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="C15" s="9" t="n">
-        <v>-20</v>
-      </c>
-      <c r="D15" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="E15" s="11" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="7" t="n">
-        <v>46293</v>
-      </c>
-      <c r="B16" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="C16" s="9" t="n">
-        <v>-16.99</v>
-      </c>
-      <c r="D16" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="E16" s="11" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="7" t="n">
-        <v>46293</v>
-      </c>
-      <c r="B17" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="C17" s="9" t="n">
-        <v>-65.02</v>
-      </c>
-      <c r="D17" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="E17" s="11" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7" t="n">
-        <v>46293</v>
-      </c>
-      <c r="B18" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="C18" s="9" t="n">
-        <v>-12.8</v>
-      </c>
-      <c r="D18" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="E18" s="11" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="7" t="n">
-        <v>46294</v>
-      </c>
-      <c r="B19" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="C19" s="9" t="n">
-        <v>-43.74</v>
-      </c>
-      <c r="D19" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="E19" s="11" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C21" s="5" t="n">
+    </row>
+    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C21" s="6" t="n">
         <f aca="false">SUM(C2:C20)</f>
         <v>-2039.36</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="10" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="7" t="n">
+    <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B23" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="8" t="n">
         <v>46287</v>
       </c>
-      <c r="B24" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="C24" s="9" t="n">
+      <c r="B24" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C24" s="10" t="n">
         <v>-21.72</v>
       </c>
-      <c r="D24" s="10" t="s">
-        <v>39</v>
+      <c r="D24" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="E24" s="11" t="s">
         <v>7</v>

</xml_diff>

<commit_message>
Update the Terra lunch note with the FBT treatment
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RHXHFGjwTVGyoJeP29asg9
</commit_message>
<xml_diff>
--- a/cards/09. DL CTS EXP SEPT 26.xlsx
+++ b/cards/09. DL CTS EXP SEPT 26.xlsx
@@ -130,7 +130,7 @@
     <t xml:space="preserve">DEWR Lunch</t>
   </si>
   <si>
-    <t xml:space="preserve">In Xero. The CTS half of the lunch (32.00) has no GST on it but the DEWR half does. Minor, 2.91.</t>
+    <t xml:space="preserve">In Xero. CTS half has no GST because account 65115 Staff Entertainment is set to GST Free. FBT treatment, not a slip. DL was travelling overnight, so his meal could go to 58130 Direct Travel with GST instead. Check with accountant.</t>
   </si>
   <si>
     <t xml:space="preserve">CAFE RISTRETTO           CANBERRA    ACT</t>
@@ -265,7 +265,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -314,16 +314,12 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -650,7 +646,7 @@
       <c r="C4" s="3" t="n">
         <v>-30.96</v>
       </c>
-      <c r="F4" s="14" t="s">
+      <c r="F4" s="12" t="s">
         <v>12</v>
       </c>
     </row>
@@ -664,7 +660,7 @@
       <c r="C5" s="3" t="n">
         <v>-25.65</v>
       </c>
-      <c r="F5" s="14" t="s">
+      <c r="F5" s="12" t="s">
         <v>12</v>
       </c>
     </row>
@@ -695,7 +691,7 @@
       <c r="C7" s="3" t="n">
         <v>-15.16</v>
       </c>
-      <c r="F7" s="14" t="s">
+      <c r="F7" s="12" t="s">
         <v>16</v>
       </c>
     </row>

</xml_diff>